<commit_message>
update: atualização de arquivo transparencia
</commit_message>
<xml_diff>
--- a/public/transparencia/financeiro/recursos-recebidos.xlsx
+++ b/public/transparencia/financeiro/recursos-recebidos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wilson Ferrari\Documents\ENTIDADES\SC MARACAI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Prestação de Contas Hospital\Prestação Federal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DA9C615-A10B-470A-93DE-65EEA4561B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD39E9A0-4AF0-4E82-8B36-4B6094D6B27D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -513,22 +513,24 @@
   <dimension ref="A1:V6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" customWidth="1"/>
+    <col min="1" max="1" width="7.5703125" customWidth="1"/>
     <col min="2" max="2" width="15.7109375" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
-    <col min="5" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="7.7109375" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" customWidth="1"/>
+    <col min="4" max="4" width="9.7109375" customWidth="1"/>
+    <col min="5" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
     <col min="9" max="12" width="15.7109375" customWidth="1"/>
-    <col min="13" max="14" width="15.7109375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.140625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="12.5703125" style="3" customWidth="1"/>
-    <col min="17" max="17" width="13.28515625" style="4" customWidth="1"/>
-    <col min="18" max="18" width="15.7109375" style="3" customWidth="1"/>
-    <col min="19" max="19" width="12.5703125" style="3" customWidth="1"/>
-    <col min="20" max="20" width="13.140625" style="3" customWidth="1"/>
-    <col min="21" max="21" width="11.28515625" style="3" customWidth="1"/>
-    <col min="22" max="22" width="12" style="3" customWidth="1"/>
+    <col min="13" max="13" width="13.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="14.42578125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.85546875" style="3" customWidth="1"/>
+    <col min="17" max="17" width="15.7109375" style="4" customWidth="1"/>
+    <col min="18" max="18" width="14" style="3" customWidth="1"/>
+    <col min="19" max="19" width="14.28515625" style="3" customWidth="1"/>
+    <col min="20" max="20" width="12.28515625" style="3" customWidth="1"/>
+    <col min="21" max="21" width="11.42578125" style="3" customWidth="1"/>
+    <col min="22" max="22" width="11.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.25">
@@ -859,13 +861,13 @@
         <v>500000</v>
       </c>
       <c r="S5" s="3">
-        <v>0</v>
+        <v>496720.35</v>
       </c>
       <c r="T5" s="3">
-        <v>0</v>
+        <v>382300</v>
       </c>
       <c r="U5" s="3">
-        <v>0</v>
+        <v>503813.98</v>
       </c>
       <c r="V5" s="3">
         <v>0</v>

</xml_diff>